<commit_message>
Add Archnetix row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6565,28 +6565,68 @@
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="21">
-      <c r="A81" s="11" t="n"/>
-      <c r="B81" s="11" t="n"/>
-      <c r="C81" s="11" t="n"/>
-      <c r="D81" s="12" t="n"/>
-      <c r="E81" s="11" t="n"/>
-      <c r="F81" s="11" t="n"/>
-      <c r="G81" s="11" t="n"/>
-      <c r="H81" s="13" t="n"/>
-      <c r="I81" s="12" t="n"/>
-      <c r="J81" s="12" t="n"/>
+      <c r="A81" s="17" t="inlineStr">
+        <is>
+          <t>Archnetix</t>
+        </is>
+      </c>
+      <c r="B81" s="17" t="inlineStr">
+        <is>
+          <t>BIM tooling / automation developer (speculative)</t>
+        </is>
+      </c>
+      <c r="C81" s="17" t="inlineStr">
+        <is>
+          <t>Islamabad, PK / Dubai, AE</t>
+        </is>
+      </c>
+      <c r="D81" s="18" t="n"/>
+      <c r="E81" s="17" t="n"/>
+      <c r="F81" s="17" t="inlineStr">
+        <is>
+          <t>Referral</t>
+        </is>
+      </c>
+      <c r="G81" s="17" t="inlineStr">
+        <is>
+          <t>https://www.archnetix.com/</t>
+        </is>
+      </c>
+      <c r="H81" s="19" t="n"/>
+      <c r="I81" s="18" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="J81" s="18" t="n"/>
       <c r="K81" s="14">
         <f>IF($H81="","",TODAY()-$H81)</f>
         <v/>
       </c>
-      <c r="L81" s="13" t="n"/>
-      <c r="M81" s="11" t="n"/>
-      <c r="N81" s="13" t="n"/>
-      <c r="O81" s="11" t="n"/>
-      <c r="P81" s="11" t="n"/>
-      <c r="Q81" s="11" t="n"/>
-      <c r="R81" s="12" t="n"/>
-      <c r="S81" s="11" t="n"/>
+      <c r="L81" s="19" t="n"/>
+      <c r="M81" s="17" t="inlineStr">
+        <is>
+          <t>Reach out to CEO via warm connection</t>
+        </is>
+      </c>
+      <c r="N81" s="19" t="n"/>
+      <c r="O81" s="17" t="n"/>
+      <c r="P81" s="17" t="n"/>
+      <c r="Q81" s="17" t="inlineStr">
+        <is>
+          <t>uae/2026_09_13_archnetix_bim_tooling</t>
+        </is>
+      </c>
+      <c r="R81" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S81" s="17" t="inlineStr">
+        <is>
+          <t>Dubai-HQ BIM services firm (Scan-to-BIM, coordination, archviz) with main production office in Bahria Town, Islamabad. They advertise no in-house software development, so the pitch is building tools/automation on top of their BIM models and data. Warm CEO connection is the route in. CV built; no message drafted yet.</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="21">
       <c r="A82" s="11" t="n"/>

</xml_diff>

<commit_message>
Retarget Archnetix CV to Islamabad office only
Moved uae/ -> pakistan/ since the target is the Islamabad office,
not Dubai. Removed the location/availability line above the Profile;
that ground is covered in the cover letter instead.
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6577,7 +6577,7 @@
       </c>
       <c r="C81" s="17" t="inlineStr">
         <is>
-          <t>Islamabad, PK / Dubai, AE</t>
+          <t>Islamabad, PK</t>
         </is>
       </c>
       <c r="D81" s="18" t="n"/>
@@ -6614,7 +6614,7 @@
       <c r="P81" s="17" t="n"/>
       <c r="Q81" s="17" t="inlineStr">
         <is>
-          <t>uae/2026_09_13_archnetix_bim_tooling</t>
+          <t>pakistan/2026_09_13_archnetix_bim_tooling</t>
         </is>
       </c>
       <c r="R81" s="18" t="inlineStr">
@@ -6624,7 +6624,7 @@
       </c>
       <c r="S81" s="17" t="inlineStr">
         <is>
-          <t>Dubai-HQ BIM services firm (Scan-to-BIM, coordination, archviz) with main production office in Bahria Town, Islamabad. They advertise no in-house software development, so the pitch is building tools/automation on top of their BIM models and data. Warm CEO connection is the route in. CV built; no message drafted yet.</t>
+          <t>Dubai-HQ BIM services firm (Scan-to-BIM, coordination, archviz) with main production office in Bahria Town, Islamabad. Targeting the Islamabad office only; user does not want the UAE. They advertise no in-house software development, so the pitch is building tools/automation on top of their BIM models and data. Warm CEO connection is the route in. CV built; no message drafted yet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FirstClass Sales Engineer row to Job Application Tracker
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6629,28 +6629,66 @@
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="21">
-      <c r="A82" s="11" t="n"/>
-      <c r="B82" s="11" t="n"/>
-      <c r="C82" s="11" t="n"/>
-      <c r="D82" s="12" t="n"/>
-      <c r="E82" s="11" t="n"/>
-      <c r="F82" s="11" t="n"/>
-      <c r="G82" s="11" t="n"/>
-      <c r="H82" s="13" t="n"/>
-      <c r="I82" s="12" t="n"/>
-      <c r="J82" s="12" t="n"/>
+      <c r="A82" s="17" t="inlineStr">
+        <is>
+          <t>FirstClass d.o.o. (recruiter)</t>
+        </is>
+      </c>
+      <c r="B82" s="17" t="inlineStr">
+        <is>
+          <t>Sales Engineer (formwork and scaffolding)</t>
+        </is>
+      </c>
+      <c r="C82" s="17" t="inlineStr">
+        <is>
+          <t>Ljubljana, SI / field across Slovenia</t>
+        </is>
+      </c>
+      <c r="D82" s="18" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="E82" s="17" t="n"/>
+      <c r="F82" s="17" t="inlineStr">
+        <is>
+          <t>Recruiter</t>
+        </is>
+      </c>
+      <c r="G82" s="17" t="n"/>
+      <c r="H82" s="19" t="n">
+        <v>46285</v>
+      </c>
+      <c r="I82" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J82" s="18" t="n"/>
       <c r="K82" s="14">
         <f>IF($H82="","",TODAY()-$H82)</f>
         <v/>
       </c>
-      <c r="L82" s="13" t="n"/>
-      <c r="M82" s="11" t="n"/>
-      <c r="N82" s="13" t="n"/>
-      <c r="O82" s="11" t="n"/>
-      <c r="P82" s="11" t="n"/>
-      <c r="Q82" s="11" t="n"/>
-      <c r="R82" s="12" t="n"/>
-      <c r="S82" s="11" t="n"/>
+      <c r="L82" s="19" t="n"/>
+      <c r="M82" s="17" t="n"/>
+      <c r="N82" s="19" t="n"/>
+      <c r="O82" s="17" t="n"/>
+      <c r="P82" s="17" t="n"/>
+      <c r="Q82" s="17" t="inlineStr">
+        <is>
+          <t>slovenia/2026_09_20_firstclass_sales_engineer</t>
+        </is>
+      </c>
+      <c r="R82" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S82" s="17" t="inlineStr">
+        <is>
+          <t>End client not named: an international formwork and scaffolding company. Career pivot toward technical sales, so the CV drops the software/AI material and leads on construction, FIDIC contract exposure and 5D cost estimation. Posting asks for 1-3 years experience. Category B licence stated on the CV; user confirmed they hold one.</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="21">
       <c r="A83" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Spar Slovenia Facilities Maintenance Coordinator row to tracker
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6691,28 +6691,66 @@
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="21">
-      <c r="A83" s="11" t="n"/>
-      <c r="B83" s="11" t="n"/>
-      <c r="C83" s="11" t="n"/>
-      <c r="D83" s="12" t="n"/>
-      <c r="E83" s="11" t="n"/>
-      <c r="F83" s="11" t="n"/>
-      <c r="G83" s="11" t="n"/>
-      <c r="H83" s="13" t="n"/>
-      <c r="I83" s="12" t="n"/>
-      <c r="J83" s="12" t="n"/>
+      <c r="A83" s="17" t="inlineStr">
+        <is>
+          <t>Spar Slovenija d.o.o.</t>
+        </is>
+      </c>
+      <c r="B83" s="17" t="inlineStr">
+        <is>
+          <t>Facilities Maintenance Coordinator</t>
+        </is>
+      </c>
+      <c r="C83" s="17" t="inlineStr">
+        <is>
+          <t>Ljubljana, SI</t>
+        </is>
+      </c>
+      <c r="D83" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E83" s="17" t="n"/>
+      <c r="F83" s="17" t="inlineStr">
+        <is>
+          <t>Job Board</t>
+        </is>
+      </c>
+      <c r="G83" s="17" t="n"/>
+      <c r="H83" s="19" t="n">
+        <v>46285</v>
+      </c>
+      <c r="I83" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J83" s="18" t="n"/>
       <c r="K83" s="14">
         <f>IF($H83="","",TODAY()-$H83)</f>
         <v/>
       </c>
-      <c r="L83" s="13" t="n"/>
-      <c r="M83" s="11" t="n"/>
-      <c r="N83" s="13" t="n"/>
-      <c r="O83" s="11" t="n"/>
-      <c r="P83" s="11" t="n"/>
-      <c r="Q83" s="11" t="n"/>
-      <c r="R83" s="12" t="n"/>
-      <c r="S83" s="11" t="n"/>
+      <c r="L83" s="19" t="n"/>
+      <c r="M83" s="17" t="n"/>
+      <c r="N83" s="19" t="n"/>
+      <c r="O83" s="17" t="n"/>
+      <c r="P83" s="17" t="n"/>
+      <c r="Q83" s="17" t="inlineStr">
+        <is>
+          <t>slovenia/2026_09_20_spar_facilities_coordinator</t>
+        </is>
+      </c>
+      <c r="R83" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S83" s="17" t="inlineStr">
+        <is>
+          <t>Centralising maintenance across 100 Spar stores and 13 Interspar centres. Education far exceeds the 5th-level minimum; energy management coursework maps to the building energy duty, 5D cost estimation to cost analyses, FIDIC internship to tenders/orders/contracts. Category B licence stated for branch inspections. Slovene A1 is the main soft risk.</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="21">
       <c r="A84" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Iskra order coordinator row to Job Application Tracker
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6753,28 +6753,66 @@
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="21">
-      <c r="A84" s="11" t="n"/>
-      <c r="B84" s="11" t="n"/>
-      <c r="C84" s="11" t="n"/>
-      <c r="D84" s="12" t="n"/>
-      <c r="E84" s="11" t="n"/>
-      <c r="F84" s="11" t="n"/>
-      <c r="G84" s="11" t="n"/>
-      <c r="H84" s="13" t="n"/>
-      <c r="I84" s="12" t="n"/>
-      <c r="J84" s="12" t="n"/>
+      <c r="A84" s="17" t="inlineStr">
+        <is>
+          <t>Iskra d.o.o.</t>
+        </is>
+      </c>
+      <c r="B84" s="17" t="inlineStr">
+        <is>
+          <t>Order and production coordinator (customers/sales/logistics link)</t>
+        </is>
+      </c>
+      <c r="C84" s="17" t="inlineStr">
+        <is>
+          <t>Slovenia (Kranj / Ljubljana area)</t>
+        </is>
+      </c>
+      <c r="D84" s="18" t="n"/>
+      <c r="E84" s="17" t="n"/>
+      <c r="F84" s="17" t="inlineStr">
+        <is>
+          <t>Job Board</t>
+        </is>
+      </c>
+      <c r="G84" s="17" t="inlineStr">
+        <is>
+          <t>https://www.iskra.si/</t>
+        </is>
+      </c>
+      <c r="H84" s="19" t="n">
+        <v>46285</v>
+      </c>
+      <c r="I84" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J84" s="18" t="n"/>
       <c r="K84" s="14">
         <f>IF($H84="","",TODAY()-$H84)</f>
         <v/>
       </c>
-      <c r="L84" s="13" t="n"/>
-      <c r="M84" s="11" t="n"/>
-      <c r="N84" s="13" t="n"/>
-      <c r="O84" s="11" t="n"/>
-      <c r="P84" s="11" t="n"/>
-      <c r="Q84" s="11" t="n"/>
-      <c r="R84" s="12" t="n"/>
-      <c r="S84" s="11" t="n"/>
+      <c r="L84" s="19" t="n"/>
+      <c r="M84" s="17" t="n"/>
+      <c r="N84" s="19" t="n"/>
+      <c r="O84" s="17" t="n"/>
+      <c r="P84" s="17" t="n"/>
+      <c r="Q84" s="17" t="inlineStr">
+        <is>
+          <t>slovenia/2026_09_20_iskra_order_coordinator</t>
+        </is>
+      </c>
+      <c r="R84" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S84" s="17" t="inlineStr">
+        <is>
+          <t>Long-shot, flagged to user before building. Posting wants economics/commerce/logistics education capped at VI/2, 1-3 years experience, and lists ERP, logistics and transport organisation as advantages, none of which the candidate has. Built on transferable coordination, FIDIC document review, process modelling and cost analysis instead.</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="21">
       <c r="A85" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sumer technical documentation row to Job Application Tracker
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6815,28 +6815,66 @@
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="21">
-      <c r="A85" s="11" t="n"/>
-      <c r="B85" s="11" t="n"/>
-      <c r="C85" s="11" t="n"/>
-      <c r="D85" s="12" t="n"/>
-      <c r="E85" s="11" t="n"/>
-      <c r="F85" s="11" t="n"/>
-      <c r="G85" s="11" t="n"/>
-      <c r="H85" s="13" t="n"/>
-      <c r="I85" s="12" t="n"/>
-      <c r="J85" s="12" t="n"/>
+      <c r="A85" s="17" t="inlineStr">
+        <is>
+          <t>Sumer d.o.o.</t>
+        </is>
+      </c>
+      <c r="B85" s="17" t="inlineStr">
+        <is>
+          <t>Technical documentation / production technologist</t>
+        </is>
+      </c>
+      <c r="C85" s="17" t="inlineStr">
+        <is>
+          <t>Slovenia</t>
+        </is>
+      </c>
+      <c r="D85" s="18" t="n"/>
+      <c r="E85" s="17" t="n"/>
+      <c r="F85" s="17" t="inlineStr">
+        <is>
+          <t>Job Board</t>
+        </is>
+      </c>
+      <c r="G85" s="17" t="inlineStr">
+        <is>
+          <t>http://www.sumer.si/</t>
+        </is>
+      </c>
+      <c r="H85" s="19" t="n">
+        <v>46285</v>
+      </c>
+      <c r="I85" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J85" s="18" t="n"/>
       <c r="K85" s="14">
         <f>IF($H85="","",TODAY()-$H85)</f>
         <v/>
       </c>
-      <c r="L85" s="13" t="n"/>
-      <c r="M85" s="11" t="n"/>
-      <c r="N85" s="13" t="n"/>
-      <c r="O85" s="11" t="n"/>
-      <c r="P85" s="11" t="n"/>
-      <c r="Q85" s="11" t="n"/>
-      <c r="R85" s="12" t="n"/>
-      <c r="S85" s="11" t="n"/>
+      <c r="L85" s="19" t="n"/>
+      <c r="M85" s="17" t="n"/>
+      <c r="N85" s="19" t="n"/>
+      <c r="O85" s="17" t="n"/>
+      <c r="P85" s="17" t="n"/>
+      <c r="Q85" s="17" t="inlineStr">
+        <is>
+          <t>slovenia/2026_09_20_sumer_technical_documentation</t>
+        </is>
+      </c>
+      <c r="R85" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S85" s="17" t="inlineStr">
+        <is>
+          <t>Long-shot, flagged before building. Plastics injection moulding manufacturer; core duties (injection programs, tool testing, first-piece approval under ISO/TS 16949, production time norms, mechanical working drawings) need mechanical/moulding training the candidate lacks. Stated expectations are only behavioural, which is the one opening. Built on document control, cost estimation, quality validation and supplier checking.</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="21">
       <c r="A86" s="11" t="n"/>

</xml_diff>

<commit_message>
Add HRM Solutions Constructor row to Job Application Tracker
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6877,28 +6877,74 @@
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="21">
-      <c r="A86" s="11" t="n"/>
-      <c r="B86" s="11" t="n"/>
-      <c r="C86" s="11" t="n"/>
-      <c r="D86" s="12" t="n"/>
-      <c r="E86" s="11" t="n"/>
-      <c r="F86" s="11" t="n"/>
-      <c r="G86" s="11" t="n"/>
-      <c r="H86" s="13" t="n"/>
-      <c r="I86" s="12" t="n"/>
-      <c r="J86" s="12" t="n"/>
+      <c r="A86" s="17" t="inlineStr">
+        <is>
+          <t>HRM solutions d.o.o. (recruiter)</t>
+        </is>
+      </c>
+      <c r="B86" s="17" t="inlineStr">
+        <is>
+          <t>Constructor / mechanical design engineer (aerospace client)</t>
+        </is>
+      </c>
+      <c r="C86" s="17" t="inlineStr">
+        <is>
+          <t>Slovenia</t>
+        </is>
+      </c>
+      <c r="D86" s="18" t="n"/>
+      <c r="E86" s="17" t="inlineStr">
+        <is>
+          <t>EUR 2,200 - 2,500 gross/month</t>
+        </is>
+      </c>
+      <c r="F86" s="17" t="inlineStr">
+        <is>
+          <t>Recruiter</t>
+        </is>
+      </c>
+      <c r="G86" s="17" t="inlineStr">
+        <is>
+          <t>https://hrm-resitve.si/</t>
+        </is>
+      </c>
+      <c r="H86" s="19" t="n">
+        <v>46285</v>
+      </c>
+      <c r="I86" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J86" s="18" t="n"/>
       <c r="K86" s="14">
         <f>IF($H86="","",TODAY()-$H86)</f>
         <v/>
       </c>
-      <c r="L86" s="13" t="n"/>
-      <c r="M86" s="11" t="n"/>
-      <c r="N86" s="13" t="n"/>
-      <c r="O86" s="11" t="n"/>
-      <c r="P86" s="11" t="n"/>
-      <c r="Q86" s="11" t="n"/>
-      <c r="R86" s="12" t="n"/>
-      <c r="S86" s="11" t="n"/>
+      <c r="L86" s="19" t="n"/>
+      <c r="M86" s="17" t="inlineStr">
+        <is>
+          <t>Consider a separate speculative registration with this agency for BIM/construction roles</t>
+        </is>
+      </c>
+      <c r="N86" s="19" t="n"/>
+      <c r="O86" s="17" t="n"/>
+      <c r="P86" s="17" t="n"/>
+      <c r="Q86" s="17" t="inlineStr">
+        <is>
+          <t>slovenia/2026_09_20_hrm_solutions_constructor</t>
+        </is>
+      </c>
+      <c r="R86" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S86" s="17" t="inlineStr">
+        <is>
+          <t>Weakest fit of the 20 Sep batch, flagged before building. Posting explicitly requires a mechanical engineering degree and states 3 years experience as mandatory; salary band indicates they are buying experience. End client is in aerospace. Built on 3D modelling from 2D drawings, quantity take-off as BOM analog, and document approval workflows. Agency is worth a separate speculative approach in the candidate's actual field.</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="21">
       <c r="A87" s="11" t="n"/>

</xml_diff>

<commit_message>
Add SZ-Infrastruktura NOC GSM-R row to Job Application Tracker
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6947,28 +6947,72 @@
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="21">
-      <c r="A87" s="11" t="n"/>
-      <c r="B87" s="11" t="n"/>
-      <c r="C87" s="11" t="n"/>
-      <c r="D87" s="12" t="n"/>
-      <c r="E87" s="11" t="n"/>
-      <c r="F87" s="11" t="n"/>
-      <c r="G87" s="11" t="n"/>
-      <c r="H87" s="13" t="n"/>
-      <c r="I87" s="12" t="n"/>
-      <c r="J87" s="12" t="n"/>
+      <c r="A87" s="17" t="inlineStr">
+        <is>
+          <t>SZ-Infrastruktura d.o.o. (Slovenske zeleznice)</t>
+        </is>
+      </c>
+      <c r="B87" s="17" t="inlineStr">
+        <is>
+          <t>Professional Associate I, NOC GSM-R supervision (ref. 180/26)</t>
+        </is>
+      </c>
+      <c r="C87" s="17" t="inlineStr">
+        <is>
+          <t>Ljubljana, SI</t>
+        </is>
+      </c>
+      <c r="D87" s="18" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="E87" s="17" t="n"/>
+      <c r="F87" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G87" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sz.si/kariera/</t>
+        </is>
+      </c>
+      <c r="H87" s="19" t="n">
+        <v>46285</v>
+      </c>
+      <c r="I87" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J87" s="18" t="n"/>
       <c r="K87" s="14">
         <f>IF($H87="","",TODAY()-$H87)</f>
         <v/>
       </c>
-      <c r="L87" s="13" t="n"/>
-      <c r="M87" s="11" t="n"/>
-      <c r="N87" s="13" t="n"/>
-      <c r="O87" s="11" t="n"/>
-      <c r="P87" s="11" t="n"/>
-      <c r="Q87" s="11" t="n"/>
-      <c r="R87" s="12" t="n"/>
-      <c r="S87" s="11" t="n"/>
+      <c r="L87" s="19" t="n"/>
+      <c r="M87" s="17" t="n"/>
+      <c r="N87" s="19" t="n">
+        <v>46288</v>
+      </c>
+      <c r="O87" s="17" t="n"/>
+      <c r="P87" s="17" t="n"/>
+      <c r="Q87" s="17" t="inlineStr">
+        <is>
+          <t>slovenia/2026_09_20_sz_infrastruktura_noc_gsmr</t>
+        </is>
+      </c>
+      <c r="R87" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S87" s="17" t="inlineStr">
+        <is>
+          <t>Posting deadline 23 Sep 2026; 2 positions. Best of the 20 Sep batch after Spar: education condition says relevant field with electrical engineering only preferred, experience bar is 12 months, and selected candidates are trained for the telecoms technician qualification. Hooks: maintenance process coordination/optimisation and technical bases for tenders. Gaps: no telecom/EE background, no 12 months similar experience. Fixed-term 1 year with 4-month probation.</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="21">
       <c r="A88" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Mercor AI safety red team row to Job Application Tracker
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -7015,28 +7015,70 @@
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="21">
-      <c r="A88" s="11" t="n"/>
-      <c r="B88" s="11" t="n"/>
-      <c r="C88" s="11" t="n"/>
-      <c r="D88" s="12" t="n"/>
-      <c r="E88" s="11" t="n"/>
-      <c r="F88" s="11" t="n"/>
-      <c r="G88" s="11" t="n"/>
-      <c r="H88" s="13" t="n"/>
-      <c r="I88" s="12" t="n"/>
-      <c r="J88" s="12" t="n"/>
+      <c r="A88" s="17" t="inlineStr">
+        <is>
+          <t>Mercor</t>
+        </is>
+      </c>
+      <c r="B88" s="17" t="inlineStr">
+        <is>
+          <t>AI Safety Expert, red teaming (English &amp; Urdu)</t>
+        </is>
+      </c>
+      <c r="C88" s="17" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D88" s="18" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E88" s="17" t="inlineStr">
+        <is>
+          <t>USD 16 - 22/hour, contractor</t>
+        </is>
+      </c>
+      <c r="F88" s="17" t="inlineStr">
+        <is>
+          <t>Job Board</t>
+        </is>
+      </c>
+      <c r="G88" s="17" t="n"/>
+      <c r="H88" s="19" t="n">
+        <v>46295</v>
+      </c>
+      <c r="I88" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J88" s="18" t="n"/>
       <c r="K88" s="14">
         <f>IF($H88="","",TODAY()-$H88)</f>
         <v/>
       </c>
-      <c r="L88" s="13" t="n"/>
-      <c r="M88" s="11" t="n"/>
-      <c r="N88" s="13" t="n"/>
-      <c r="O88" s="11" t="n"/>
-      <c r="P88" s="11" t="n"/>
-      <c r="Q88" s="11" t="n"/>
-      <c r="R88" s="12" t="n"/>
-      <c r="S88" s="11" t="n"/>
+      <c r="L88" s="19" t="n"/>
+      <c r="M88" s="17" t="n"/>
+      <c r="N88" s="19" t="n"/>
+      <c r="O88" s="17" t="n"/>
+      <c r="P88" s="17" t="n"/>
+      <c r="Q88" s="17" t="inlineStr">
+        <is>
+          <t>remote/2026_09_30_mercor_ai_safety_red_team</t>
+        </is>
+      </c>
+      <c r="R88" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S88" s="17" t="inlineStr">
+        <is>
+          <t>Best substantive fit to date: the MSc thesis is itself a systematic LLM evaluation study (validated judge, matched conditions, 23 datasets, 367 questions, prompt-design ablation), which is the methodology this role wants. Urdu native fluency is the hard gate and was confirmed for the first time on this date. English corrected to C2 from the understated C1 used on all prior CVs. Gaps: no formal red teaming or cybersecurity background, both listed only as nice-to-have. Independent contractor engagement, weekly Stripe/Wise.</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="21">
       <c r="A89" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Brickborne speculative row to Job Application Tracker
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -7081,28 +7081,76 @@
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="21">
-      <c r="A89" s="11" t="n"/>
-      <c r="B89" s="11" t="n"/>
-      <c r="C89" s="11" t="n"/>
-      <c r="D89" s="12" t="n"/>
-      <c r="E89" s="11" t="n"/>
-      <c r="F89" s="11" t="n"/>
-      <c r="G89" s="11" t="n"/>
-      <c r="H89" s="13" t="n"/>
-      <c r="I89" s="12" t="n"/>
-      <c r="J89" s="12" t="n"/>
+      <c r="A89" s="17" t="inlineStr">
+        <is>
+          <t>Brickborne</t>
+        </is>
+      </c>
+      <c r="B89" s="17" t="inlineStr">
+        <is>
+          <t>BIM specialist / Revit modelling (speculative, no posting)</t>
+        </is>
+      </c>
+      <c r="C89" s="17" t="inlineStr">
+        <is>
+          <t>California, USA (remote)</t>
+        </is>
+      </c>
+      <c r="D89" s="18" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E89" s="17" t="n"/>
+      <c r="F89" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G89" s="17" t="inlineStr">
+        <is>
+          <t>https://brickborne.com/</t>
+        </is>
+      </c>
+      <c r="H89" s="19" t="n"/>
+      <c r="I89" s="18" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="J89" s="18" t="n"/>
       <c r="K89" s="14">
         <f>IF($H89="","",TODAY()-$H89)</f>
         <v/>
       </c>
-      <c r="L89" s="13" t="n"/>
-      <c r="M89" s="11" t="n"/>
-      <c r="N89" s="13" t="n"/>
-      <c r="O89" s="11" t="n"/>
-      <c r="P89" s="11" t="n"/>
-      <c r="Q89" s="11" t="n"/>
-      <c r="R89" s="12" t="n"/>
-      <c r="S89" s="11" t="n"/>
+      <c r="L89" s="19" t="n"/>
+      <c r="M89" s="17" t="inlineStr">
+        <is>
+          <t>Send speculative outreach to founder Hamza Khan (shared NUST alma mater)</t>
+        </is>
+      </c>
+      <c r="N89" s="19" t="n"/>
+      <c r="O89" s="17" t="inlineStr">
+        <is>
+          <t>Hamza Khan (founder/CEO)</t>
+        </is>
+      </c>
+      <c r="P89" s="17" t="n"/>
+      <c r="Q89" s="17" t="inlineStr">
+        <is>
+          <t>usa/2026_10_08_brickborne_bim_specialist</t>
+        </is>
+      </c>
+      <c r="R89" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S89" s="17" t="inlineStr">
+        <is>
+          <t>Small founder-led drafting/BIM firm, no careers page, so speculative. Services: permit drawings, construction documentation, CAD drafting, BIM modelling, scan-to-BIM, MEP/HVAC drawings, rendering, quantity surveying. Stack Revit/AutoCAD/Navisworks. Founder Hamza Khan is a NUST civil engineering graduate, same alma mater, which is the warm hook for outreach. Gaps: no Navisworks and no rendering/visualisation tools, both left unclaimed. CV built; outreach message not yet written.</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="21">
       <c r="A90" s="11" t="n"/>

</xml_diff>